<commit_message>
"The changes hasbeen pushed to Amazon Dyanamic"
</commit_message>
<xml_diff>
--- a/src/test/resources/Excel/Updated.xlsx
+++ b/src/test/resources/Excel/Updated.xlsx
@@ -1,22 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27932"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28227"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lenovo\git\NewOneUpdated\src\test\resources\Excel\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4960A917-EF56-4136-B80E-D880F1A21D47}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{6E49FDEC-998B-49E9-B29C-EA23F483F571}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="RUNMANAGER" sheetId="1" r:id="rId1"/>
     <sheet name="DATA" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="0"/>
+  <oleSize ref="A1:J18"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -26,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="18">
   <si>
     <t>testname</t>
   </si>
@@ -43,27 +39,12 @@
     <t>count</t>
   </si>
   <si>
-    <t>loginLogoutTest</t>
-  </si>
-  <si>
-    <t>To check whether the user can sucessfully login and logout</t>
-  </si>
-  <si>
     <t>Yes</t>
   </si>
   <si>
-    <t>newTest</t>
-  </si>
-  <si>
-    <t>To check whether this test is executed</t>
-  </si>
-  <si>
     <t>1</t>
   </si>
   <si>
-    <t>2</t>
-  </si>
-  <si>
     <t>username</t>
   </si>
   <si>
@@ -76,25 +57,25 @@
     <t>yes</t>
   </si>
   <si>
-    <t>no</t>
-  </si>
-  <si>
-    <t>Admin</t>
-  </si>
-  <si>
-    <t>admin123</t>
-  </si>
-  <si>
-    <t xml:space="preserve">amunathan </t>
-  </si>
-  <si>
-    <t>testing mini bytes</t>
-  </si>
-  <si>
-    <t>subscribe</t>
-  </si>
-  <si>
     <t/>
+  </si>
+  <si>
+    <t>amazonTest</t>
+  </si>
+  <si>
+    <t>To check the amazon page is working</t>
+  </si>
+  <si>
+    <t>menutext</t>
+  </si>
+  <si>
+    <t>Laptops</t>
+  </si>
+  <si>
+    <t>browser</t>
+  </si>
+  <si>
+    <t>chrome</t>
   </si>
 </sst>
 </file>
@@ -419,7 +400,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16.42578125" customWidth="1"/>
@@ -444,37 +425,20 @@
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
+      <c r="A2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C2" t="s">
         <v>5</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="D2" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>10</v>
-      </c>
       <c r="E2" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
     </row>
   </sheetData>
@@ -484,7 +448,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DC414C53-8916-4505-A028-5436F01C0B74}">
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:G2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20.140625" customWidth="1"/>
@@ -492,9 +456,10 @@
     <col min="3" max="3" width="15.28515625" customWidth="1"/>
     <col min="4" max="4" width="14" customWidth="1"/>
     <col min="5" max="5" width="19.140625" customWidth="1"/>
+    <col min="6" max="6" width="12.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -502,98 +467,42 @@
         <v>2</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="G1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
         <v>12</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
-        <v>5</v>
-      </c>
       <c r="B2" s="1" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>17</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>18</v>
+        <v>11</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B4" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="G2" s="1" t="s">
         <v>15</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="E5" s="1" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="E6" s="1" t="s">
-        <v>21</v>
       </c>
     </row>
   </sheetData>

</xml_diff>